<commit_message>
Update rank 2026-09-13 07:20
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C456"/>
+  <dimension ref="A1:C457"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7820,6 +7820,23 @@
         </is>
       </c>
     </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-09-13 07:18</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-13 13:45
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C457"/>
+  <dimension ref="A1:C458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7837,6 +7837,23 @@
         </is>
       </c>
     </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:43</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-14 07:45
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C458"/>
+  <dimension ref="A1:C459"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7854,6 +7854,23 @@
         </is>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:43</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-14 15:48
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C459"/>
+  <dimension ref="A1:C460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7871,6 +7871,23 @@
         </is>
       </c>
     </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-09-14 15:46</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-15 07:29
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C460"/>
+  <dimension ref="A1:C461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7888,6 +7888,23 @@
         </is>
       </c>
     </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:27</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-15 14:16
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C461"/>
+  <dimension ref="A1:C462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7905,6 +7905,23 @@
         </is>
       </c>
     </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-09-15 14:14</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-16 07:28
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C462"/>
+  <dimension ref="A1:C463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7922,6 +7922,23 @@
         </is>
       </c>
     </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:26</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-16 14:08
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C463"/>
+  <dimension ref="A1:C464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7939,6 +7939,23 @@
         </is>
       </c>
     </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:06</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-17 07:25
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C464"/>
+  <dimension ref="A1:C465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7956,6 +7956,23 @@
         </is>
       </c>
     </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:23</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-17 14:14
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C465"/>
+  <dimension ref="A1:C466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7973,6 +7973,23 @@
         </is>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:12</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-18 07:14
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C466"/>
+  <dimension ref="A1:C467"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7990,6 +7990,23 @@
         </is>
       </c>
     </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:12</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-18 13:32
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C467"/>
+  <dimension ref="A1:C468"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8007,6 +8007,23 @@
         </is>
       </c>
     </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:30</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-19 07:12
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C468"/>
+  <dimension ref="A1:C469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8024,6 +8024,23 @@
         </is>
       </c>
     </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-09-19 07:10</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-19 13:00
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C469"/>
+  <dimension ref="A1:C470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8041,6 +8041,23 @@
         </is>
       </c>
     </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-09-19 12:58</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-20 07:37
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C470"/>
+  <dimension ref="A1:C471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8058,6 +8058,23 @@
         </is>
       </c>
     </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-09-20 07:35</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-20 13:32
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C471"/>
+  <dimension ref="A1:C472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8075,6 +8075,23 @@
         </is>
       </c>
     </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-09-20 13:30</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-21 07:49
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C472"/>
+  <dimension ref="A1:C473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8092,6 +8092,23 @@
         </is>
       </c>
     </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:47</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-21 15:47
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C473"/>
+  <dimension ref="A1:C474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8109,6 +8109,23 @@
         </is>
       </c>
     </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:46</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-22 07:32
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C474"/>
+  <dimension ref="A1:C475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8126,6 +8126,23 @@
         </is>
       </c>
     </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:30</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-22 13:59
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C475"/>
+  <dimension ref="A1:C476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8143,6 +8143,23 @@
         </is>
       </c>
     </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-09-22 13:57</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-23 07:35
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C476"/>
+  <dimension ref="A1:C477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8160,6 +8160,23 @@
         </is>
       </c>
     </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:33</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-23 14:10
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C477"/>
+  <dimension ref="A1:C478"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8177,6 +8177,23 @@
         </is>
       </c>
     </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:08</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-24 07:27
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C478"/>
+  <dimension ref="A1:C479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8194,6 +8194,23 @@
         </is>
       </c>
     </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:25</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-24 14:08
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C479"/>
+  <dimension ref="A1:C480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8211,6 +8211,23 @@
         </is>
       </c>
     </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:06</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-25 07:24
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C480"/>
+  <dimension ref="A1:C481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8228,6 +8228,23 @@
         </is>
       </c>
     </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:21</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-25 14:31
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C481"/>
+  <dimension ref="A1:C482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8245,6 +8245,23 @@
         </is>
       </c>
     </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:29</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-26 07:19
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C482"/>
+  <dimension ref="A1:C483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8262,6 +8262,23 @@
         </is>
       </c>
     </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-09-26 07:17</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-26 13:42
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C483"/>
+  <dimension ref="A1:C484"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8279,6 +8279,23 @@
         </is>
       </c>
     </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:40</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-27 07:51
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C484"/>
+  <dimension ref="A1:C485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8296,6 +8296,23 @@
         </is>
       </c>
     </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-09-27 07:49</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-27 14:38
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C485"/>
+  <dimension ref="A1:C486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8313,6 +8313,23 @@
         </is>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:36</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-28 08:28
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C486"/>
+  <dimension ref="A1:C487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8330,6 +8330,23 @@
         </is>
       </c>
     </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-09-28 08:26</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-28 17:31
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C487"/>
+  <dimension ref="A1:C488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8347,6 +8347,23 @@
         </is>
       </c>
     </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:28</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-29 08:08
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C488"/>
+  <dimension ref="A1:C489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8364,6 +8364,23 @@
         </is>
       </c>
     </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-09-29 08:06</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-29 15:33
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C489"/>
+  <dimension ref="A1:C490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8381,6 +8381,23 @@
         </is>
       </c>
     </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:31</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-30 08:14
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C490"/>
+  <dimension ref="A1:C491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8398,6 +8398,23 @@
         </is>
       </c>
     </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-09-30 08:12</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-09-30 15:46
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C491"/>
+  <dimension ref="A1:C492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8415,6 +8415,23 @@
         </is>
       </c>
     </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:44</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-01 08:36
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C492"/>
+  <dimension ref="A1:C493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8432,6 +8432,23 @@
         </is>
       </c>
     </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-10-01 08:34</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-01 16:11
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C493"/>
+  <dimension ref="A1:C494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8449,6 +8449,23 @@
         </is>
       </c>
     </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:09</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-02 08:12
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C494"/>
+  <dimension ref="A1:C495"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8466,6 +8466,23 @@
         </is>
       </c>
     </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-10-02 08:09</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-02 15:35
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C495"/>
+  <dimension ref="A1:C496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8483,6 +8483,23 @@
         </is>
       </c>
     </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:33</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-03 07:50
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C496"/>
+  <dimension ref="A1:C497"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8500,6 +8500,23 @@
         </is>
       </c>
     </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-10-03 07:47</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-03 14:13
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C497"/>
+  <dimension ref="A1:C498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8517,6 +8517,23 @@
         </is>
       </c>
     </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:11</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-04 07:58
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C498"/>
+  <dimension ref="A1:C499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8534,6 +8534,23 @@
         </is>
       </c>
     </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-10-04 07:56</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-04 14:44
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C499"/>
+  <dimension ref="A1:C500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8551,6 +8551,23 @@
         </is>
       </c>
     </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:42</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-05 08:41
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C500"/>
+  <dimension ref="A1:C501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8568,6 +8568,23 @@
         </is>
       </c>
     </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-10-05 08:39</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-05 18:11
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C501"/>
+  <dimension ref="A1:C502"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8585,6 +8585,23 @@
         </is>
       </c>
     </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:08</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-06 08:47
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C502"/>
+  <dimension ref="A1:C503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8602,6 +8602,23 @@
         </is>
       </c>
     </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-10-06 08:44</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-06 15:47
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C503"/>
+  <dimension ref="A1:C504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8619,6 +8619,23 @@
         </is>
       </c>
     </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:46</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-07 08:21
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C504"/>
+  <dimension ref="A1:C505"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8636,6 +8636,23 @@
         </is>
       </c>
     </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-10-07 08:19</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-07 16:13
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C505"/>
+  <dimension ref="A1:C506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8653,6 +8653,23 @@
         </is>
       </c>
     </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:11</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-08 08:37
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C506"/>
+  <dimension ref="A1:C507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8670,6 +8670,23 @@
         </is>
       </c>
     </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:35</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-08 16:14
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C507"/>
+  <dimension ref="A1:C508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8687,6 +8687,23 @@
         </is>
       </c>
     </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:12</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-09 08:43
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C508"/>
+  <dimension ref="A1:C509"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8704,6 +8704,23 @@
         </is>
       </c>
     </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-10-09 08:41</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-09 15:58
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C509"/>
+  <dimension ref="A1:C510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8721,6 +8721,23 @@
         </is>
       </c>
     </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-10-09 15:56</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-10 08:17
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C510"/>
+  <dimension ref="A1:C511"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8738,6 +8738,23 @@
         </is>
       </c>
     </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-10-10 08:15</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-10 15:09
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C511"/>
+  <dimension ref="A1:C512"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8755,6 +8755,23 @@
         </is>
       </c>
     </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:07</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-11 08:32
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C512"/>
+  <dimension ref="A1:C513"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8772,6 +8772,23 @@
         </is>
       </c>
     </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-10-11 08:30</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-11 15:28
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C513"/>
+  <dimension ref="A1:C514"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8789,6 +8789,23 @@
         </is>
       </c>
     </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:26</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-12 08:52
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C514"/>
+  <dimension ref="A1:C515"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8806,6 +8806,23 @@
         </is>
       </c>
     </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-10-12 08:51</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-12 18:48
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C515"/>
+  <dimension ref="A1:C516"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8823,6 +8823,23 @@
         </is>
       </c>
     </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-10-12 18:46</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-13 09:09
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C516"/>
+  <dimension ref="A1:C517"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8840,6 +8840,23 @@
         </is>
       </c>
     </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-10-13 09:07</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-14 07:19
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C517"/>
+  <dimension ref="A1:C518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8857,6 +8857,23 @@
         </is>
       </c>
     </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:17</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-14 14:26
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C518"/>
+  <dimension ref="A1:C519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8874,6 +8874,23 @@
         </is>
       </c>
     </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:24</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-15 07:11
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C519"/>
+  <dimension ref="A1:C520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8891,6 +8891,23 @@
         </is>
       </c>
     </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-10-15 07:09</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-15 14:03
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C520"/>
+  <dimension ref="A1:C521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8908,6 +8908,23 @@
         </is>
       </c>
     </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:01</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-16 06:54
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C521"/>
+  <dimension ref="A1:C522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8925,6 +8925,23 @@
         </is>
       </c>
     </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-10-16 06:52</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-16 13:51
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C522"/>
+  <dimension ref="A1:C523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8942,6 +8942,23 @@
         </is>
       </c>
     </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-10-16 13:49</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-17 06:46
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C523"/>
+  <dimension ref="A1:C524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8959,6 +8959,23 @@
         </is>
       </c>
     </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-10-17 06:44</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-17 12:48
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C524"/>
+  <dimension ref="A1:C525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8976,6 +8976,23 @@
         </is>
       </c>
     </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-10-17 12:46</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-18 07:05
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C525"/>
+  <dimension ref="A1:C526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8993,6 +8993,23 @@
         </is>
       </c>
     </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-10-18 07:04</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-18 13:07
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C526"/>
+  <dimension ref="A1:C527"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9010,6 +9010,23 @@
         </is>
       </c>
     </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-10-18 13:05</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-19 07:31
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C527"/>
+  <dimension ref="A1:C528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9027,6 +9027,23 @@
         </is>
       </c>
     </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:29</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-19 16:20
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C528"/>
+  <dimension ref="A1:C529"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9044,6 +9044,23 @@
         </is>
       </c>
     </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-10-19 16:18</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-20 07:20
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C529"/>
+  <dimension ref="A1:C530"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9061,6 +9061,23 @@
         </is>
       </c>
     </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:18</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-20 14:13
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C530"/>
+  <dimension ref="A1:C531"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9078,6 +9078,23 @@
         </is>
       </c>
     </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:11</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-21 07:19
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C531"/>
+  <dimension ref="A1:C532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9095,6 +9095,23 @@
         </is>
       </c>
     </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-10-21 07:17</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-21 14:25
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C532"/>
+  <dimension ref="A1:C533"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9112,6 +9112,23 @@
         </is>
       </c>
     </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:23</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-22 07:20
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C533"/>
+  <dimension ref="A1:C534"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9129,6 +9129,23 @@
         </is>
       </c>
     </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:18</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-22 14:27
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C534"/>
+  <dimension ref="A1:C535"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9146,6 +9146,23 @@
         </is>
       </c>
     </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:25</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-23 07:13
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C535"/>
+  <dimension ref="A1:C536"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9163,6 +9163,23 @@
         </is>
       </c>
     </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-10-23 07:11</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-23 14:09
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C536"/>
+  <dimension ref="A1:C537"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9180,6 +9180,23 @@
         </is>
       </c>
     </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-10-23 14:07</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-24 07:02
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C537"/>
+  <dimension ref="A1:C538"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9197,6 +9197,23 @@
         </is>
       </c>
     </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-10-24 07:00</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-24 13:12
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C538"/>
+  <dimension ref="A1:C539"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9214,6 +9214,23 @@
         </is>
       </c>
     </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-10-24 13:10</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-25 07:27
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C539"/>
+  <dimension ref="A1:C540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9231,6 +9231,23 @@
         </is>
       </c>
     </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-10-25 07:25</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-25 13:39
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C540"/>
+  <dimension ref="A1:C541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9248,6 +9248,23 @@
         </is>
       </c>
     </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-10-25 13:37</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-26 07:36
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C541"/>
+  <dimension ref="A1:C542"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9265,6 +9265,23 @@
         </is>
       </c>
     </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:34</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-26 16:00
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C542"/>
+  <dimension ref="A1:C543"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9282,6 +9282,23 @@
         </is>
       </c>
     </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-10-26 15:58</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-27 07:33
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C543"/>
+  <dimension ref="A1:C544"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9299,6 +9299,23 @@
         </is>
       </c>
     </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-10-27 07:31</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-27 15:14
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C544"/>
+  <dimension ref="A1:C545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9316,6 +9316,23 @@
         </is>
       </c>
     </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-10-27 15:12</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-28 08:05
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C545"/>
+  <dimension ref="A1:C546"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9333,6 +9333,23 @@
         </is>
       </c>
     </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-10-28 08:03</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-28 15:50
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C546"/>
+  <dimension ref="A1:C547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9350,6 +9350,23 @@
         </is>
       </c>
     </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-10-28 15:48</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-29 08:15
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C547"/>
+  <dimension ref="A1:C548"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9367,6 +9367,23 @@
         </is>
       </c>
     </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-10-29 08:13</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-29 15:58
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C548"/>
+  <dimension ref="A1:C549"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9384,6 +9384,23 @@
         </is>
       </c>
     </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-10-29 15:56</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-30 08:21
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C549"/>
+  <dimension ref="A1:C550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9401,6 +9401,23 @@
         </is>
       </c>
     </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-10-30 08:19</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-30 15:44
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C550"/>
+  <dimension ref="A1:C551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9418,6 +9418,23 @@
         </is>
       </c>
     </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-10-30 15:42</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-31 08:11
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C551"/>
+  <dimension ref="A1:C552"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9435,6 +9435,23 @@
         </is>
       </c>
     </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-10-31 08:09</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update rank 2026-10-31 15:13
</commit_message>
<xml_diff>
--- a/플레이스_순위_통합기록.xlsx
+++ b/플레이스_순위_통합기록.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C552"/>
+  <dimension ref="A1:C553"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9452,6 +9452,23 @@
         </is>
       </c>
     </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-10-31 15:11</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>순위권 밖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>